<commit_message>
daily auto push: 2026-09-13 12:41 UTC
</commit_message>
<xml_diff>
--- a/excel/spotify.xlsx
+++ b/excel/spotify.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D844"/>
+  <dimension ref="A1:D845"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15519,16 +15519,16 @@
     <row r="839">
       <c r="A839" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/09/12</t>
         </is>
       </c>
       <c r="B839" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C839" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D839" t="n">
         <v>101</v>
@@ -15537,12 +15537,12 @@
     <row r="840">
       <c r="A840" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B840" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C840" t="n">
@@ -15555,12 +15555,12 @@
     <row r="841">
       <c r="A841" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B841" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C841" t="n">
@@ -15573,12 +15573,12 @@
     <row r="842">
       <c r="A842" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B842" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C842" t="n">
@@ -15591,12 +15591,12 @@
     <row r="843">
       <c r="A843" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B843" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C843" t="n">
@@ -15609,18 +15609,36 @@
     <row r="844">
       <c r="A844" t="inlineStr">
         <is>
+          <t>2027/01/02</t>
+        </is>
+      </c>
+      <c r="B844" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="C844" t="n">
+        <v>22</v>
+      </c>
+      <c r="D844" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" t="inlineStr">
+        <is>
           <t>2027/01/03</t>
         </is>
       </c>
-      <c r="B844" t="inlineStr">
+      <c r="B845" t="inlineStr">
         <is>
           <t>日</t>
         </is>
       </c>
-      <c r="C844" t="n">
-        <v>22</v>
-      </c>
-      <c r="D844" t="n">
+      <c r="C845" t="n">
+        <v>22</v>
+      </c>
+      <c r="D845" t="n">
         <v>101</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-09-15 12:38 UTC
</commit_message>
<xml_diff>
--- a/excel/spotify.xlsx
+++ b/excel/spotify.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D846"/>
+  <dimension ref="A1:D847"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15555,16 +15555,16 @@
     <row r="841">
       <c r="A841" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/09/14</t>
         </is>
       </c>
       <c r="B841" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C841" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D841" t="n">
         <v>101</v>
@@ -15573,12 +15573,12 @@
     <row r="842">
       <c r="A842" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B842" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C842" t="n">
@@ -15591,12 +15591,12 @@
     <row r="843">
       <c r="A843" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B843" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C843" t="n">
@@ -15609,12 +15609,12 @@
     <row r="844">
       <c r="A844" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B844" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C844" t="n">
@@ -15627,12 +15627,12 @@
     <row r="845">
       <c r="A845" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B845" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C845" t="n">
@@ -15645,18 +15645,36 @@
     <row r="846">
       <c r="A846" t="inlineStr">
         <is>
+          <t>2027/01/02</t>
+        </is>
+      </c>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="C846" t="n">
+        <v>22</v>
+      </c>
+      <c r="D846" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" t="inlineStr">
+        <is>
           <t>2027/01/03</t>
         </is>
       </c>
-      <c r="B846" t="inlineStr">
+      <c r="B847" t="inlineStr">
         <is>
           <t>日</t>
         </is>
       </c>
-      <c r="C846" t="n">
-        <v>22</v>
-      </c>
-      <c r="D846" t="n">
+      <c r="C847" t="n">
+        <v>22</v>
+      </c>
+      <c r="D847" t="n">
         <v>101</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-09-16 12:34 UTC
</commit_message>
<xml_diff>
--- a/excel/spotify.xlsx
+++ b/excel/spotify.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D847"/>
+  <dimension ref="A1:D848"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15573,7 +15573,7 @@
     <row r="842">
       <c r="A842" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/09/15</t>
         </is>
       </c>
       <c r="B842" t="inlineStr">
@@ -15582,7 +15582,7 @@
         </is>
       </c>
       <c r="C842" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D842" t="n">
         <v>101</v>
@@ -15591,12 +15591,12 @@
     <row r="843">
       <c r="A843" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B843" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C843" t="n">
@@ -15609,12 +15609,12 @@
     <row r="844">
       <c r="A844" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B844" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C844" t="n">
@@ -15627,12 +15627,12 @@
     <row r="845">
       <c r="A845" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B845" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C845" t="n">
@@ -15645,12 +15645,12 @@
     <row r="846">
       <c r="A846" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B846" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C846" t="n">
@@ -15663,18 +15663,36 @@
     <row r="847">
       <c r="A847" t="inlineStr">
         <is>
+          <t>2027/01/02</t>
+        </is>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="C847" t="n">
+        <v>22</v>
+      </c>
+      <c r="D847" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" t="inlineStr">
+        <is>
           <t>2027/01/03</t>
         </is>
       </c>
-      <c r="B847" t="inlineStr">
+      <c r="B848" t="inlineStr">
         <is>
           <t>日</t>
         </is>
       </c>
-      <c r="C847" t="n">
-        <v>22</v>
-      </c>
-      <c r="D847" t="n">
+      <c r="C848" t="n">
+        <v>22</v>
+      </c>
+      <c r="D848" t="n">
         <v>101</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-09-18 12:12 UTC
</commit_message>
<xml_diff>
--- a/excel/spotify.xlsx
+++ b/excel/spotify.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D849"/>
+  <dimension ref="A1:D850"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15609,16 +15609,16 @@
     <row r="844">
       <c r="A844" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/09/17</t>
         </is>
       </c>
       <c r="B844" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C844" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D844" t="n">
         <v>101</v>
@@ -15627,12 +15627,12 @@
     <row r="845">
       <c r="A845" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B845" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C845" t="n">
@@ -15645,12 +15645,12 @@
     <row r="846">
       <c r="A846" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B846" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C846" t="n">
@@ -15663,12 +15663,12 @@
     <row r="847">
       <c r="A847" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B847" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C847" t="n">
@@ -15681,12 +15681,12 @@
     <row r="848">
       <c r="A848" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B848" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C848" t="n">
@@ -15699,18 +15699,36 @@
     <row r="849">
       <c r="A849" t="inlineStr">
         <is>
+          <t>2027/01/02</t>
+        </is>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="C849" t="n">
+        <v>22</v>
+      </c>
+      <c r="D849" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" t="inlineStr">
+        <is>
           <t>2027/01/03</t>
         </is>
       </c>
-      <c r="B849" t="inlineStr">
+      <c r="B850" t="inlineStr">
         <is>
           <t>日</t>
         </is>
       </c>
-      <c r="C849" t="n">
-        <v>22</v>
-      </c>
-      <c r="D849" t="n">
+      <c r="C850" t="n">
+        <v>22</v>
+      </c>
+      <c r="D850" t="n">
         <v>101</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-09-20 12:16 UTC
</commit_message>
<xml_diff>
--- a/excel/spotify.xlsx
+++ b/excel/spotify.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D851"/>
+  <dimension ref="A1:D852"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15645,16 +15645,16 @@
     <row r="846">
       <c r="A846" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/09/19</t>
         </is>
       </c>
       <c r="B846" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C846" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D846" t="n">
         <v>101</v>
@@ -15663,12 +15663,12 @@
     <row r="847">
       <c r="A847" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B847" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C847" t="n">
@@ -15681,12 +15681,12 @@
     <row r="848">
       <c r="A848" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B848" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C848" t="n">
@@ -15699,12 +15699,12 @@
     <row r="849">
       <c r="A849" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B849" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C849" t="n">
@@ -15717,12 +15717,12 @@
     <row r="850">
       <c r="A850" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B850" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C850" t="n">
@@ -15735,18 +15735,36 @@
     <row r="851">
       <c r="A851" t="inlineStr">
         <is>
+          <t>2027/01/02</t>
+        </is>
+      </c>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="C851" t="n">
+        <v>22</v>
+      </c>
+      <c r="D851" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" t="inlineStr">
+        <is>
           <t>2027/01/03</t>
         </is>
       </c>
-      <c r="B851" t="inlineStr">
+      <c r="B852" t="inlineStr">
         <is>
           <t>日</t>
         </is>
       </c>
-      <c r="C851" t="n">
-        <v>22</v>
-      </c>
-      <c r="D851" t="n">
+      <c r="C852" t="n">
+        <v>22</v>
+      </c>
+      <c r="D852" t="n">
         <v>101</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-09-22 12:33 UTC
</commit_message>
<xml_diff>
--- a/excel/spotify.xlsx
+++ b/excel/spotify.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D853"/>
+  <dimension ref="A1:D854"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15681,16 +15681,16 @@
     <row r="848">
       <c r="A848" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/09/21</t>
         </is>
       </c>
       <c r="B848" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C848" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D848" t="n">
         <v>101</v>
@@ -15699,12 +15699,12 @@
     <row r="849">
       <c r="A849" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B849" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C849" t="n">
@@ -15717,12 +15717,12 @@
     <row r="850">
       <c r="A850" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B850" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C850" t="n">
@@ -15735,12 +15735,12 @@
     <row r="851">
       <c r="A851" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B851" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C851" t="n">
@@ -15753,12 +15753,12 @@
     <row r="852">
       <c r="A852" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B852" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C852" t="n">
@@ -15771,18 +15771,36 @@
     <row r="853">
       <c r="A853" t="inlineStr">
         <is>
+          <t>2027/01/02</t>
+        </is>
+      </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="C853" t="n">
+        <v>22</v>
+      </c>
+      <c r="D853" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" t="inlineStr">
+        <is>
           <t>2027/01/03</t>
         </is>
       </c>
-      <c r="B853" t="inlineStr">
+      <c r="B854" t="inlineStr">
         <is>
           <t>日</t>
         </is>
       </c>
-      <c r="C853" t="n">
-        <v>22</v>
-      </c>
-      <c r="D853" t="n">
+      <c r="C854" t="n">
+        <v>22</v>
+      </c>
+      <c r="D854" t="n">
         <v>101</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-09-24 12:42 UTC
</commit_message>
<xml_diff>
--- a/excel/spotify.xlsx
+++ b/excel/spotify.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D855"/>
+  <dimension ref="A1:D856"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15717,16 +15717,16 @@
     <row r="850">
       <c r="A850" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/09/23</t>
         </is>
       </c>
       <c r="B850" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C850" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D850" t="n">
         <v>101</v>
@@ -15735,12 +15735,12 @@
     <row r="851">
       <c r="A851" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B851" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C851" t="n">
@@ -15753,12 +15753,12 @@
     <row r="852">
       <c r="A852" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B852" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C852" t="n">
@@ -15771,12 +15771,12 @@
     <row r="853">
       <c r="A853" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B853" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C853" t="n">
@@ -15789,12 +15789,12 @@
     <row r="854">
       <c r="A854" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B854" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C854" t="n">
@@ -15807,18 +15807,36 @@
     <row r="855">
       <c r="A855" t="inlineStr">
         <is>
+          <t>2027/01/02</t>
+        </is>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="C855" t="n">
+        <v>22</v>
+      </c>
+      <c r="D855" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" t="inlineStr">
+        <is>
           <t>2027/01/03</t>
         </is>
       </c>
-      <c r="B855" t="inlineStr">
+      <c r="B856" t="inlineStr">
         <is>
           <t>日</t>
         </is>
       </c>
-      <c r="C855" t="n">
-        <v>22</v>
-      </c>
-      <c r="D855" t="n">
+      <c r="C856" t="n">
+        <v>22</v>
+      </c>
+      <c r="D856" t="n">
         <v>101</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-09-26 12:12 UTC
</commit_message>
<xml_diff>
--- a/excel/spotify.xlsx
+++ b/excel/spotify.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D857"/>
+  <dimension ref="A1:D858"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15753,16 +15753,16 @@
     <row r="852">
       <c r="A852" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/09/26</t>
         </is>
       </c>
       <c r="B852" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C852" t="n">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="D852" t="n">
         <v>101</v>
@@ -15771,12 +15771,12 @@
     <row r="853">
       <c r="A853" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B853" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C853" t="n">
@@ -15789,12 +15789,12 @@
     <row r="854">
       <c r="A854" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B854" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C854" t="n">
@@ -15807,12 +15807,12 @@
     <row r="855">
       <c r="A855" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B855" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C855" t="n">
@@ -15825,12 +15825,12 @@
     <row r="856">
       <c r="A856" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B856" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C856" t="n">
@@ -15843,18 +15843,36 @@
     <row r="857">
       <c r="A857" t="inlineStr">
         <is>
+          <t>2027/01/02</t>
+        </is>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="C857" t="n">
+        <v>22</v>
+      </c>
+      <c r="D857" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" t="inlineStr">
+        <is>
           <t>2027/01/03</t>
         </is>
       </c>
-      <c r="B857" t="inlineStr">
+      <c r="B858" t="inlineStr">
         <is>
           <t>日</t>
         </is>
       </c>
-      <c r="C857" t="n">
-        <v>22</v>
-      </c>
-      <c r="D857" t="n">
+      <c r="C858" t="n">
+        <v>22</v>
+      </c>
+      <c r="D858" t="n">
         <v>101</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-10-15 12:37 UTC
</commit_message>
<xml_diff>
--- a/excel/spotify.xlsx
+++ b/excel/spotify.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D876"/>
+  <dimension ref="A1:D877"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16095,16 +16095,16 @@
     <row r="871">
       <c r="A871" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/10/14</t>
         </is>
       </c>
       <c r="B871" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C871" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D871" t="n">
         <v>101</v>
@@ -16113,12 +16113,12 @@
     <row r="872">
       <c r="A872" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B872" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C872" t="n">
@@ -16131,12 +16131,12 @@
     <row r="873">
       <c r="A873" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B873" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C873" t="n">
@@ -16149,12 +16149,12 @@
     <row r="874">
       <c r="A874" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B874" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C874" t="n">
@@ -16167,12 +16167,12 @@
     <row r="875">
       <c r="A875" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B875" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C875" t="n">
@@ -16185,18 +16185,36 @@
     <row r="876">
       <c r="A876" t="inlineStr">
         <is>
+          <t>2027/01/02</t>
+        </is>
+      </c>
+      <c r="B876" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="C876" t="n">
+        <v>22</v>
+      </c>
+      <c r="D876" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" t="inlineStr">
+        <is>
           <t>2027/01/03</t>
         </is>
       </c>
-      <c r="B876" t="inlineStr">
+      <c r="B877" t="inlineStr">
         <is>
           <t>日</t>
         </is>
       </c>
-      <c r="C876" t="n">
-        <v>22</v>
-      </c>
-      <c r="D876" t="n">
+      <c r="C877" t="n">
+        <v>22</v>
+      </c>
+      <c r="D877" t="n">
         <v>101</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-10-16 12:20 UTC
</commit_message>
<xml_diff>
--- a/excel/spotify.xlsx
+++ b/excel/spotify.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D877"/>
+  <dimension ref="A1:D878"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16113,16 +16113,16 @@
     <row r="872">
       <c r="A872" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/10/15</t>
         </is>
       </c>
       <c r="B872" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C872" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D872" t="n">
         <v>101</v>
@@ -16131,12 +16131,12 @@
     <row r="873">
       <c r="A873" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B873" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C873" t="n">
@@ -16149,12 +16149,12 @@
     <row r="874">
       <c r="A874" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B874" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C874" t="n">
@@ -16167,12 +16167,12 @@
     <row r="875">
       <c r="A875" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B875" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C875" t="n">
@@ -16185,12 +16185,12 @@
     <row r="876">
       <c r="A876" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B876" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C876" t="n">
@@ -16203,18 +16203,36 @@
     <row r="877">
       <c r="A877" t="inlineStr">
         <is>
+          <t>2027/01/02</t>
+        </is>
+      </c>
+      <c r="B877" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="C877" t="n">
+        <v>22</v>
+      </c>
+      <c r="D877" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" t="inlineStr">
+        <is>
           <t>2027/01/03</t>
         </is>
       </c>
-      <c r="B877" t="inlineStr">
+      <c r="B878" t="inlineStr">
         <is>
           <t>日</t>
         </is>
       </c>
-      <c r="C877" t="n">
-        <v>22</v>
-      </c>
-      <c r="D877" t="n">
+      <c r="C878" t="n">
+        <v>22</v>
+      </c>
+      <c r="D878" t="n">
         <v>101</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-10-19 13:00 UTC
</commit_message>
<xml_diff>
--- a/excel/spotify.xlsx
+++ b/excel/spotify.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D880"/>
+  <dimension ref="A1:D881"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16167,16 +16167,16 @@
     <row r="875">
       <c r="A875" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/10/18</t>
         </is>
       </c>
       <c r="B875" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C875" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D875" t="n">
         <v>101</v>
@@ -16185,12 +16185,12 @@
     <row r="876">
       <c r="A876" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B876" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C876" t="n">
@@ -16203,12 +16203,12 @@
     <row r="877">
       <c r="A877" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B877" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C877" t="n">
@@ -16221,12 +16221,12 @@
     <row r="878">
       <c r="A878" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B878" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C878" t="n">
@@ -16239,12 +16239,12 @@
     <row r="879">
       <c r="A879" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B879" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C879" t="n">
@@ -16257,18 +16257,36 @@
     <row r="880">
       <c r="A880" t="inlineStr">
         <is>
+          <t>2027/01/02</t>
+        </is>
+      </c>
+      <c r="B880" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="C880" t="n">
+        <v>22</v>
+      </c>
+      <c r="D880" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" t="inlineStr">
+        <is>
           <t>2027/01/03</t>
         </is>
       </c>
-      <c r="B880" t="inlineStr">
+      <c r="B881" t="inlineStr">
         <is>
           <t>日</t>
         </is>
       </c>
-      <c r="C880" t="n">
-        <v>22</v>
-      </c>
-      <c r="D880" t="n">
+      <c r="C881" t="n">
+        <v>22</v>
+      </c>
+      <c r="D881" t="n">
         <v>101</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-10-20 12:41 UTC
</commit_message>
<xml_diff>
--- a/excel/spotify.xlsx
+++ b/excel/spotify.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D881"/>
+  <dimension ref="A1:D882"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16185,16 +16185,16 @@
     <row r="876">
       <c r="A876" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/10/19</t>
         </is>
       </c>
       <c r="B876" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C876" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D876" t="n">
         <v>101</v>
@@ -16203,12 +16203,12 @@
     <row r="877">
       <c r="A877" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B877" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C877" t="n">
@@ -16221,12 +16221,12 @@
     <row r="878">
       <c r="A878" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B878" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C878" t="n">
@@ -16239,12 +16239,12 @@
     <row r="879">
       <c r="A879" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B879" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C879" t="n">
@@ -16257,12 +16257,12 @@
     <row r="880">
       <c r="A880" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B880" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C880" t="n">
@@ -16275,18 +16275,36 @@
     <row r="881">
       <c r="A881" t="inlineStr">
         <is>
+          <t>2027/01/02</t>
+        </is>
+      </c>
+      <c r="B881" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="C881" t="n">
+        <v>22</v>
+      </c>
+      <c r="D881" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" t="inlineStr">
+        <is>
           <t>2027/01/03</t>
         </is>
       </c>
-      <c r="B881" t="inlineStr">
+      <c r="B882" t="inlineStr">
         <is>
           <t>日</t>
         </is>
       </c>
-      <c r="C881" t="n">
-        <v>22</v>
-      </c>
-      <c r="D881" t="n">
+      <c r="C882" t="n">
+        <v>22</v>
+      </c>
+      <c r="D882" t="n">
         <v>101</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-10-21 12:53 UTC
</commit_message>
<xml_diff>
--- a/excel/spotify.xlsx
+++ b/excel/spotify.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D882"/>
+  <dimension ref="A1:D883"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16203,7 +16203,7 @@
     <row r="877">
       <c r="A877" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/10/20</t>
         </is>
       </c>
       <c r="B877" t="inlineStr">
@@ -16212,7 +16212,7 @@
         </is>
       </c>
       <c r="C877" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D877" t="n">
         <v>101</v>
@@ -16221,12 +16221,12 @@
     <row r="878">
       <c r="A878" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B878" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C878" t="n">
@@ -16239,12 +16239,12 @@
     <row r="879">
       <c r="A879" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B879" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C879" t="n">
@@ -16257,12 +16257,12 @@
     <row r="880">
       <c r="A880" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B880" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C880" t="n">
@@ -16275,12 +16275,12 @@
     <row r="881">
       <c r="A881" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B881" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C881" t="n">
@@ -16293,18 +16293,36 @@
     <row r="882">
       <c r="A882" t="inlineStr">
         <is>
+          <t>2027/01/02</t>
+        </is>
+      </c>
+      <c r="B882" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="C882" t="n">
+        <v>22</v>
+      </c>
+      <c r="D882" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" t="inlineStr">
+        <is>
           <t>2027/01/03</t>
         </is>
       </c>
-      <c r="B882" t="inlineStr">
+      <c r="B883" t="inlineStr">
         <is>
           <t>日</t>
         </is>
       </c>
-      <c r="C882" t="n">
-        <v>22</v>
-      </c>
-      <c r="D882" t="n">
+      <c r="C883" t="n">
+        <v>22</v>
+      </c>
+      <c r="D883" t="n">
         <v>101</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-10-23 12:35 UTC
</commit_message>
<xml_diff>
--- a/excel/spotify.xlsx
+++ b/excel/spotify.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D884"/>
+  <dimension ref="A1:D885"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16239,16 +16239,16 @@
     <row r="879">
       <c r="A879" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/10/22</t>
         </is>
       </c>
       <c r="B879" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C879" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D879" t="n">
         <v>101</v>
@@ -16257,12 +16257,12 @@
     <row r="880">
       <c r="A880" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B880" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C880" t="n">
@@ -16275,12 +16275,12 @@
     <row r="881">
       <c r="A881" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B881" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C881" t="n">
@@ -16293,12 +16293,12 @@
     <row r="882">
       <c r="A882" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B882" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C882" t="n">
@@ -16311,12 +16311,12 @@
     <row r="883">
       <c r="A883" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B883" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C883" t="n">
@@ -16329,18 +16329,36 @@
     <row r="884">
       <c r="A884" t="inlineStr">
         <is>
+          <t>2027/01/02</t>
+        </is>
+      </c>
+      <c r="B884" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="C884" t="n">
+        <v>22</v>
+      </c>
+      <c r="D884" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" t="inlineStr">
+        <is>
           <t>2027/01/03</t>
         </is>
       </c>
-      <c r="B884" t="inlineStr">
+      <c r="B885" t="inlineStr">
         <is>
           <t>日</t>
         </is>
       </c>
-      <c r="C884" t="n">
-        <v>22</v>
-      </c>
-      <c r="D884" t="n">
+      <c r="C885" t="n">
+        <v>22</v>
+      </c>
+      <c r="D885" t="n">
         <v>101</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-10-25 12:31 UTC
</commit_message>
<xml_diff>
--- a/excel/spotify.xlsx
+++ b/excel/spotify.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D886"/>
+  <dimension ref="A1:D887"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16275,16 +16275,16 @@
     <row r="881">
       <c r="A881" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/10/24</t>
         </is>
       </c>
       <c r="B881" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C881" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D881" t="n">
         <v>101</v>
@@ -16293,12 +16293,12 @@
     <row r="882">
       <c r="A882" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B882" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C882" t="n">
@@ -16311,12 +16311,12 @@
     <row r="883">
       <c r="A883" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B883" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C883" t="n">
@@ -16329,12 +16329,12 @@
     <row r="884">
       <c r="A884" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B884" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C884" t="n">
@@ -16347,12 +16347,12 @@
     <row r="885">
       <c r="A885" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B885" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C885" t="n">
@@ -16365,18 +16365,36 @@
     <row r="886">
       <c r="A886" t="inlineStr">
         <is>
+          <t>2027/01/02</t>
+        </is>
+      </c>
+      <c r="B886" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="C886" t="n">
+        <v>22</v>
+      </c>
+      <c r="D886" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" t="inlineStr">
+        <is>
           <t>2027/01/03</t>
         </is>
       </c>
-      <c r="B886" t="inlineStr">
+      <c r="B887" t="inlineStr">
         <is>
           <t>日</t>
         </is>
       </c>
-      <c r="C886" t="n">
-        <v>22</v>
-      </c>
-      <c r="D886" t="n">
+      <c r="C887" t="n">
+        <v>22</v>
+      </c>
+      <c r="D887" t="n">
         <v>101</v>
       </c>
     </row>

</xml_diff>